<commit_message>
Actualiza plantilla de impresion
</commit_message>
<xml_diff>
--- a/templates/trazabilidad de prenda 1.xlsx
+++ b/templates/trazabilidad de prenda 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/54afb4c87f83e63f/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cristel/Desktop/provisional/backend/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4CC03993-4B83-4673-9D37-C940842ED59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFE245B3-49CD-FF4E-9EAC-E6A858A72E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{3985ED2D-E0E6-427C-853C-5C7E8C730A94}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15840" xr2:uid="{3985ED2D-E0E6-427C-853C-5C7E8C730A94}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
   <si>
     <t>PEDIDO</t>
   </si>
@@ -69,7 +69,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -271,6 +271,15 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -283,23 +292,14 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -689,197 +689,6 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>493513</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="28" name="Imagen 27">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C0B4D3D-74EA-469B-929C-2BC75AD1204D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1524000" y="4352925"/>
-          <a:ext cx="4465438" cy="542925"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>26604</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="CuadroTexto 29">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2A2415A-35F7-4144-8763-A3C0C96E870C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3095625" y="4933950"/>
-          <a:ext cx="1255329" cy="295275"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="FFFF00"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="es-MX" sz="1100"/>
-            <a:t>TARJETA KANBAN</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>523875</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>670832</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>68036</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="CuadroTexto 30">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AC84E016-7B2D-4E11-AB17-DBEBBB17A881}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6019800" y="5019675"/>
-          <a:ext cx="908957" cy="163286"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:schemeClr val="lt1">
-              <a:shade val="50000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:r>
-            <a:rPr lang="es-MX" sz="1100"/>
-            <a:t>Folio:______</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
@@ -940,115 +749,6 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>400707</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>183931</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>755431</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>6569</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="33" name="Conector recto 32">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B33770F-8D50-4BD2-BBC7-8E087F739355}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1924707" y="3965356"/>
-          <a:ext cx="5088649" cy="13138"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>742950</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>115942</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="34" name="CuadroTexto 33">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{612F2BC9-D2F8-4743-863D-FCC0116C06D3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="742950" y="5105400"/>
-          <a:ext cx="6276975" cy="4287892"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="es-MX" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1428,283 +1128,149 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B6:K40"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <dimension ref="B6:K17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="12.140625" customWidth="1"/>
-    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" customWidth="1"/>
+    <col min="4" max="4" width="11.5" customWidth="1"/>
     <col min="5" max="5" width="6" customWidth="1"/>
-    <col min="6" max="6" width="6.42578125" customWidth="1"/>
-    <col min="7" max="7" width="5.85546875" customWidth="1"/>
-    <col min="8" max="8" width="6.140625" customWidth="1"/>
+    <col min="6" max="6" width="6.5" customWidth="1"/>
+    <col min="7" max="7" width="5.83203125" customWidth="1"/>
+    <col min="8" max="8" width="6.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:11" ht="18.75">
+    <row r="6" spans="2:11" ht="19" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="16" t="s">
+      <c r="E6" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="16"/>
-      <c r="G6" s="16" t="s">
+      <c r="F6" s="7"/>
+      <c r="G6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H6" s="16"/>
+      <c r="H6" s="7"/>
       <c r="I6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:11" ht="24">
+    <row r="7" spans="2:11" ht="24" x14ac:dyDescent="0.3">
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="12"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="9"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="9" spans="2:11">
-      <c r="C9" s="14" t="s">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="C9" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="I9" s="15" t="s">
+      <c r="D9" s="16"/>
+      <c r="I9" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="J9" s="15"/>
+      <c r="J9" s="14"/>
     </row>
-    <row r="10" spans="2:11" ht="24">
-      <c r="C10" s="11"/>
-      <c r="D10" s="12"/>
+    <row r="10" spans="2:11" ht="24" x14ac:dyDescent="0.3">
+      <c r="C10" s="8"/>
+      <c r="D10" s="9"/>
       <c r="E10" s="3"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="12"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="9"/>
     </row>
-    <row r="11" spans="2:11" ht="15" customHeight="1">
-      <c r="B11" s="13" t="s">
+    <row r="11" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+      <c r="K11" s="15"/>
     </row>
-    <row r="12" spans="2:11" ht="24">
+    <row r="12" spans="2:11" ht="24" x14ac:dyDescent="0.3">
       <c r="B12" s="5"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="13"/>
       <c r="I12" s="6"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
     </row>
-    <row r="13" spans="2:11" ht="24">
+    <row r="13" spans="2:11" ht="24" x14ac:dyDescent="0.3">
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="12"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="9"/>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
     </row>
-    <row r="14" spans="2:11">
-      <c r="B14" s="13" t="s">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B14" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+      <c r="K14" s="15"/>
     </row>
-    <row r="15" spans="2:11" ht="24">
+    <row r="15" spans="2:11" ht="24" x14ac:dyDescent="0.3">
       <c r="B15" s="5"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="13"/>
       <c r="I15" s="6"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="2:11" ht="24">
+    <row r="16" spans="2:11" ht="24" x14ac:dyDescent="0.3">
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="12"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="9"/>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="2:10">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="29" spans="2:10" ht="18.75">
-      <c r="C29" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16" t="s">
-        <v>3</v>
-      </c>
-      <c r="H29" s="16"/>
-      <c r="I29" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="2:10" ht="24">
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="12"/>
-      <c r="I30" s="2"/>
-    </row>
-    <row r="32" spans="2:10">
-      <c r="C32" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="14"/>
-      <c r="I32" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="J32" s="15"/>
-    </row>
-    <row r="33" spans="2:11" ht="24">
-      <c r="C33" s="11"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="3"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="12"/>
-    </row>
-    <row r="34" spans="2:11">
-      <c r="B34" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C34" s="13"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="13"/>
-      <c r="J34" s="13"/>
-      <c r="K34" s="13"/>
-    </row>
-    <row r="35" spans="2:11" ht="24">
-      <c r="B35" s="5"/>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-    </row>
-    <row r="36" spans="2:11" ht="24">
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="12"/>
-      <c r="I36" s="2"/>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-    </row>
-    <row r="37" spans="2:11">
-      <c r="B37" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="13"/>
-      <c r="J37" s="13"/>
-      <c r="K37" s="13"/>
-    </row>
-    <row r="38" spans="2:11" ht="24">
-      <c r="B38" s="5"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="10"/>
-      <c r="I38" s="6"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-    </row>
-    <row r="39" spans="2:11" ht="24">
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="12"/>
-      <c r="I39" s="2"/>
-      <c r="J39" s="2"/>
-      <c r="K39" s="2"/>
-    </row>
-    <row r="40" spans="2:11">
-      <c r="B40" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="36">
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="G12:H12"/>
+  <mergeCells count="18">
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:J10"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="G29:H29"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="G13:H13"/>
     <mergeCell ref="B11:K11"/>
@@ -1713,22 +1279,12 @@
     <mergeCell ref="G15:H15"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="I32:J32"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="I33:J33"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="E39:F39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="B34:K34"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="B37:K37"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="G12:H12"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>